<commit_message>
chore: strip Read Me and Benchmark tabs from exercise fixtures
Ann asked (2026-09-25) that the public repo describe the data only as
fictional profiles shaped by overall percentages. Both committed
workbooks now hold only the Profiles and Events sheets.

1. SmartMatch_Student_Body_300.xlsx: Read Me and Benchmark removed.
2. SmartMatch_Student_Body_Sample_20.xlsx: Read Me removed.
3. Document properties reset; custom properties and names of removed
   sheets dropped. No comments existed.
4. Every Profiles and Events cell is identical (openpyxl, data_only).
5. Test docstrings that quoted Read Me lines now state the fact in their
   own words and cite "Ann's data file, 2026-09-24". No test logic
   changed; 2 test functions renamed away from "read_me".

Tabs removed going forward; earlier copies remain in git history by
owner decision.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/exercise/SmartMatch_Student_Body_Sample_20.xlsx
+++ b/tests/fixtures/exercise/SmartMatch_Student_Body_Sample_20.xlsx
@@ -1,19 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profiles" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Profiles" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Events" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Profiles'!$A$1:$N$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Events'!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Profiles'!$A$1:$N$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Events'!$A$1:$H$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -464,361 +463,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Smart Match — made-up student body (20-row sample)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Prepared by Dr. Ann Wang for the Smart Match team, Sept 24, 2026. For the AI in Marketing class exercise.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Every row is fictional. No real student appears in this file. Names were made up and checked against the survey list so none matches a real respondent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Column names are final. The sample is 20 rows taken from the full file (same IDs, same values).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Pink columns are HIDDEN: the app must never show them and never use them for matching.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Topics use one fixed list of 13 fields (the same list as the 2026 Fall Career Readiness Survey).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Profiles sheet — columns</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>profile_id</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Unique ID for each made-up profile (P001–P300). Never changes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>first_name</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Made-up first name. Fictional; no real student.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>last_name</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Made-up last name. Fictional; no real student.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>major</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Major. Always known. Used by the "same major" factor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Freshman, Sophomore, Junior or Senior. Used in the tie-break (seniors first).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>events_attended</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Past event IDs attended (E01–E10), separated by ";". Blank = none. Used by "went to similar events before".</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>events_attended_count</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Number of past events attended (0–5).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>card_completed</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Yes/No: has this profile filled in the profile card? About 70 say Yes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>stated_interests</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Topics the profile said it is interested in (card holders only), separated by ";". Blank if no card. Used by "said they are interested".</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>stated_career_goal</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Career goal from the profile card. Blank if no card. Used by "career goal fits this event".</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>info_level</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>"How much we know" marker: Major only / Major + events attended / Completed card. Can also be computed by the app from the columns above.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>tiebreak_order</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Fixed random order 1–300 for the last step of the tie-break. Never changes between runs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>hidden_true_interests</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>HIDDEN. The profile's real interests. Never shown and never used for matching. Used only by the results rule and by the refresh (a new card copies these).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>hidden_true_career_goal</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>HIDDEN. The profile's real career goal. Same rules as hidden_true_interests.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Events sheet — columns</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>event_id</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>E01–E10 are past events (attendance history). E11 and E12 are the two exercise events.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>event_name</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Made-up event name. Companies are fictional.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>event_type</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Kind of event.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>event_date</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Date (past events 2025–26; exercise dates are placeholders).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>event_topics</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Topics, separated by ";", using the same topic list as the profiles.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>target_major</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>The major the organizer aims at. Used by "same major".</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>exercise_event</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Yes for E11 (Northline) and E12 (Harbor).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>seats</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Seats for the exercise events (60).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>Test case</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>P004 is an Accounting major whose card states an interest in Technology / information systems. For the Northline event (E11), with "said they are interested" turned up, it should rank above a plain Accounting major; with it turned off, it should not.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2140,7 +1784,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>